<commit_message>
BOM, schematic and assembly drawing generated
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Voltage_3V3_5V/Rev02/BOM/BOM_JLC-UZ_D_Voltage_3V3_5V(Default).xlsx
+++ b/Project Outputs for UZ_D_Voltage_3V3_5V/Rev02/BOM/BOM_JLC-UZ_D_Voltage_3V3_5V(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\uz_d_voltage_3v3_5v\Project Outputs for UZ_D_Voltage_3V3_5V\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB2FFA84-92C3-4946-88EB-90B867B5B805}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DDA9F13-6FC5-438F-81ED-1A6757532A95}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22830" windowHeight="12405" xr2:uid="{4BB3FDDF-9CA8-41F3-B7EC-A56159D57A00}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13965" xr2:uid="{6223F1D5-FA57-4276-B9A0-31E26CC788FD}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Voltage_3V3_5V(Def" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="151">
   <si>
     <t>Quantity</t>
   </si>
@@ -84,6 +84,27 @@
     <t>UZgen_C_0603_100nF_50V_X7R</t>
   </si>
   <si>
+    <t>1 µF</t>
+  </si>
+  <si>
+    <t>C13, C15</t>
+  </si>
+  <si>
+    <t>16V</t>
+  </si>
+  <si>
+    <t>UZgen_C_0603_1uF_16V_X7R</t>
+  </si>
+  <si>
+    <t>220 nF</t>
+  </si>
+  <si>
+    <t>C14</t>
+  </si>
+  <si>
+    <t>UZgen_C_0603_220nF_50V_X7R</t>
+  </si>
+  <si>
     <t>150060BS84000</t>
   </si>
   <si>
@@ -234,7 +255,7 @@
     <t>0R</t>
   </si>
   <si>
-    <t>R42, R73, R74, R76, R77</t>
+    <t>R76, R77</t>
   </si>
   <si>
     <t>UZgen_R_0603_0R</t>
@@ -835,8 +856,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A5A0388-1DAC-4947-8790-3059C7A43C2D}">
-  <dimension ref="A1:K26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{795E0A02-377D-4DBA-B0AE-057118900D90}">
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -919,7 +940,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>18</v>
@@ -928,321 +949,325 @@
         <v>19</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>23</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="1"/>
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="I4" s="1"/>
       <c r="J4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>30</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="K4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="E5" s="1"/>
       <c r="F5" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>37</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="I7" s="1"/>
       <c r="J7" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="K7" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="K8" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K9" s="1"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>63</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="K11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="K12" s="1"/>
+      <c r="K12" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K13" s="1"/>
     </row>
@@ -1251,27 +1276,27 @@
         <v>2</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K14" s="1"/>
     </row>
@@ -1280,152 +1305,148 @@
         <v>1</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>84</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="K16" s="1"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>1</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>89</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>91</v>
-      </c>
+      <c r="K17" s="1"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>1</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -1433,61 +1454,61 @@
         <v>1</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="2" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1495,59 +1516,61 @@
         <v>1</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E23" s="1"/>
+        <v>121</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="F23" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K23" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1555,30 +1578,30 @@
         <v>1</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -1586,54 +1609,114 @@
         <v>1</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="K25" s="1"/>
+        <v>132</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>1</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="2" t="s">
-        <v>142</v>
-      </c>
       <c r="G26" s="2" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="K26" s="1"/>
+        <v>137</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="K27" s="1"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>1</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E28" s="1"/>
+      <c r="F28" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="K28" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
- pull-down resistors at n.c. ports of fourth level shifter - set all pull-downs at VCCB side from DNP to pollute
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Voltage_3V3_5V/Rev02/BOM/BOM_JLC-UZ_D_Voltage_3V3_5V(Default).xlsx
+++ b/Project Outputs for UZ_D_Voltage_3V3_5V/Rev02/BOM/BOM_JLC-UZ_D_Voltage_3V3_5V(Default).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\uz_d_voltage_3v3_5v\Project Outputs for UZ_D_Voltage_3V3_5V\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DDA9F13-6FC5-438F-81ED-1A6757532A95}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3DE32AB-4990-4EC8-A80D-4803D32D1C37}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13965" xr2:uid="{6223F1D5-FA57-4276-B9A0-31E26CC788FD}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="17025" xr2:uid="{7B736804-B156-48A4-A676-CA63B15CA46A}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_D_Voltage_3V3_5V(Def" sheetId="1" r:id="rId1"/>
@@ -192,7 +192,7 @@
     <t>10k</t>
   </si>
   <si>
-    <t>R2, R39, R40, R41, R43, R44, R45, R46, R47, R48, R49, R50, R51, R52, R53, R54, R55, R56, R57, R58, R59, R60, R61, R62, R63, R64, R65, R66, R67, R68, R69, R70, R71, R72, R75, R78, R79, R80</t>
+    <t>R2, R39, R40, R41, R42, R43, R44, R45, R46, R47, R48, R49, R50, R51, R52, R53, R54, R55, R56, R57, R58, R59, R60, R61, R62, R63, R64, R65, R66, R67, R68, R69, R70, R71, R72, R73, R74, R75, R78, R79, R80, R85, R86, R87, R88, R89, R90, R91, R92, R93, R94, R95, R96, R97, R98, R99, R100, R101, R102, R103, R104, R105, R106, R107, R108, R109, R110, R111, R112, R113, R114, R115</t>
   </si>
   <si>
     <t>Generic resistor</t>
@@ -856,7 +856,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{795E0A02-377D-4DBA-B0AE-057118900D90}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04DD5012-EACE-4749-B2E4-E3593C0A2CB2}">
   <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1126,7 +1126,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>53</v>

</xml_diff>